<commit_message>
docs: comparacao de resultados
</commit_message>
<xml_diff>
--- a/04-backpropagation-funcao/docs/Anotações-Testes.xlsx
+++ b/04-backpropagation-funcao/docs/Anotações-Testes.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
   <si>
     <t>Bateria de Testes</t>
   </si>
@@ -86,10 +86,22 @@
     <t>58,35 s</t>
   </si>
   <si>
-    <t>0.255104</t>
-  </si>
-  <si>
     <t>58,42 s</t>
+  </si>
+  <si>
+    <t>58,51 s</t>
+  </si>
+  <si>
+    <t>58,80 s</t>
+  </si>
+  <si>
+    <t>8,36 s</t>
+  </si>
+  <si>
+    <t>25,10 s</t>
+  </si>
+  <si>
+    <t>117,03 s</t>
   </si>
 </sst>
 </file>
@@ -1660,62 +1672,142 @@
       <c r="G12" s="12">
         <v>42</v>
       </c>
-      <c r="H12" s="12" t="s">
+      <c r="H12" s="12">
+        <v>0.255104</v>
+      </c>
+      <c r="I12" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="I12" s="12" t="s">
+    </row>
+    <row r="13" spans="2:15">
+      <c r="B13" s="15">
+        <v>10</v>
+      </c>
+      <c r="C13" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="D13" s="15">
+        <v>0</v>
+      </c>
+      <c r="E13" s="15">
+        <v>35000</v>
+      </c>
+      <c r="F13" s="15">
+        <v>0.5</v>
+      </c>
+      <c r="G13" s="15">
+        <v>42</v>
+      </c>
+      <c r="H13" s="15">
+        <v>0.001942</v>
+      </c>
+      <c r="I13" s="15" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="2:15">
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
-      <c r="H13" s="15"/>
-      <c r="I13" s="15"/>
-    </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
-      <c r="I14" s="12"/>
+      <c r="B14" s="12">
+        <v>11</v>
+      </c>
+      <c r="C14" s="12">
+        <v>0.05</v>
+      </c>
+      <c r="D14" s="12">
+        <v>0</v>
+      </c>
+      <c r="E14" s="12">
+        <v>35000</v>
+      </c>
+      <c r="F14" s="12">
+        <v>1</v>
+      </c>
+      <c r="G14" s="12">
+        <v>42</v>
+      </c>
+      <c r="H14" s="12">
+        <v>0.002302</v>
+      </c>
+      <c r="I14" s="12" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
+      <c r="B15" s="15">
+        <v>12</v>
+      </c>
+      <c r="C15" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="D15" s="15">
+        <v>0</v>
+      </c>
+      <c r="E15" s="15">
+        <v>5000</v>
+      </c>
+      <c r="F15" s="15">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G15" s="15">
+        <v>42</v>
+      </c>
+      <c r="H15" s="15">
+        <v>0.09417</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
-      <c r="I16" s="12"/>
+      <c r="B16" s="12">
+        <v>13</v>
+      </c>
+      <c r="C16" s="12">
+        <v>0.05</v>
+      </c>
+      <c r="D16" s="12">
+        <v>0</v>
+      </c>
+      <c r="E16" s="12">
+        <v>15000</v>
+      </c>
+      <c r="F16" s="12">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G16" s="12">
+        <v>42</v>
+      </c>
+      <c r="H16" s="12">
+        <v>0.006989</v>
+      </c>
+      <c r="I16" s="12" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="17" spans="2:9">
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
+      <c r="B17" s="15">
+        <v>14</v>
+      </c>
+      <c r="C17" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="D17" s="15">
+        <v>0</v>
+      </c>
+      <c r="E17" s="15">
+        <v>70000</v>
+      </c>
+      <c r="F17" s="15">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G17" s="15">
+        <v>42</v>
+      </c>
+      <c r="H17" s="15">
+        <v>0.001846</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="18" spans="2:9">
       <c r="B18" s="12"/>
@@ -1728,14 +1820,14 @@
       <c r="I18" s="12"/>
     </row>
     <row r="19" spans="2:9">
-      <c r="B19" s="15"/>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="15"/>
-      <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
-      <c r="H19" s="15"/>
-      <c r="I19" s="15"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="12"/>
@@ -1748,14 +1840,14 @@
       <c r="I20" s="12"/>
     </row>
     <row r="21" spans="2:9">
-      <c r="B21" s="15"/>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
     </row>
     <row r="22" spans="2:9">
       <c r="B22" s="12"/>

</xml_diff>

<commit_message>
docs: comparacao de sementes
</commit_message>
<xml_diff>
--- a/04-backpropagation-funcao/docs/Anotações-Testes.xlsx
+++ b/04-backpropagation-funcao/docs/Anotações-Testes.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>Bateria de Testes</t>
   </si>
@@ -102,6 +102,12 @@
   </si>
   <si>
     <t>117,03 s</t>
+  </si>
+  <si>
+    <t>117,07 s</t>
+  </si>
+  <si>
+    <t>118,86 s</t>
   </si>
 </sst>
 </file>
@@ -1810,24 +1816,56 @@
       </c>
     </row>
     <row r="18" spans="2:9">
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
-      <c r="I18" s="12"/>
+      <c r="B18" s="12">
+        <v>15</v>
+      </c>
+      <c r="C18" s="12">
+        <v>0.05</v>
+      </c>
+      <c r="D18" s="12">
+        <v>0</v>
+      </c>
+      <c r="E18" s="12">
+        <v>70000</v>
+      </c>
+      <c r="F18" s="12">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G18" s="12">
+        <v>7</v>
+      </c>
+      <c r="H18" s="12">
+        <v>0.001096</v>
+      </c>
+      <c r="I18" s="12" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="19" spans="2:9">
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
-      <c r="I19" s="12"/>
+      <c r="B19" s="15">
+        <v>16</v>
+      </c>
+      <c r="C19" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="D19" s="15">
+        <v>0</v>
+      </c>
+      <c r="E19" s="15">
+        <v>70000</v>
+      </c>
+      <c r="F19" s="15">
+        <v>0.333333333333333</v>
+      </c>
+      <c r="G19" s="15">
+        <v>123</v>
+      </c>
+      <c r="H19" s="15">
+        <v>0.000385</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="20" spans="2:9">
       <c r="B20" s="12"/>

</xml_diff>